<commit_message>
Handle SAS vs Python missing-value semantics: KB note, clarity check, '; missing if X is missing' clause
</commit_message>
<xml_diff>
--- a/examples/adam/spec_draft.xlsx
+++ b/examples/adam/spec_draft.xlsx
@@ -814,7 +814,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Set to '&lt;65' if AGE &lt; 65, else '&gt;=65'</t>
+          <t>Set to '&lt;65' if AGE &lt; 65, else '&gt;=65'; missing if AGE is missing</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -859,7 +859,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Set to 1 if AGEGR1 = '&lt;65', else 2</t>
+          <t>Set to 1 if AGEGR1 = '&lt;65', else 2; missing if AGEGR1 is missing</t>
         </is>
       </c>
       <c r="H8" t="inlineStr"/>

</xml_diff>

<commit_message>
Compiler: partial-date imputation + flag, coalesce, upcase, earliest/latest; ADAE example imputes ASTDT
</commit_message>
<xml_diff>
--- a/examples/adam/spec_draft.xlsx
+++ b/examples/adam/spec_draft.xlsx
@@ -517,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I34"/>
+  <dimension ref="A1:I35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1795,21 +1795,21 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>ASTDY</t>
+          <t>ASTDTF</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Analysis Start Relative Day</t>
+          <t>Analysis Start Date Imputation Flag</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Num</t>
+          <t>Char</t>
         </is>
       </c>
       <c r="E31" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
@@ -1818,10 +1818,14 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Study day of ASTDT relative to TRTSDT: ASTDT - TRTSDT + 1 if ASTDT &gt;= TRTSDT, else ASTDT - TRTSDT; missing if either is missing</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr"/>
+          <t>Imputation flag of AESTDTC</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>DATEFL</t>
+        </is>
+      </c>
       <c r="I31" t="inlineStr">
         <is>
           <t>Perm</t>
@@ -1836,21 +1840,21 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>TRTEMFL</t>
+          <t>ASTDY</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Treatment Emergent Analysis Flag</t>
+          <t>Analysis Start Relative Day</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Char</t>
+          <t>Num</t>
         </is>
       </c>
       <c r="E32" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
@@ -1859,34 +1863,30 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Set to 'Y' if ASTDT &gt;= ADSL.TRTSTDT</t>
-        </is>
-      </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>Study day of ASTDT relative to TRTSDT: ASTDT - TRTSDT + 1 if ASTDT &gt;= TRTSDT, else ASTDT - TRTSDT; missing if either is missing</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr">
         <is>
-          <t>Exp</t>
+          <t>Perm</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>ADSL</t>
+          <t>ADAE</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>EOSSTT</t>
+          <t>TRTEMFL</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>End of Study Status</t>
+          <t>Treatment Emergent Analysis Flag</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1895,61 +1895,106 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
           <t>Derived</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr"/>
-      <c r="H33" t="inlineStr"/>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Set to 'Y' if ASTDT &gt;= ADSL.TRTSTDT</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>Perm</t>
+          <t>Exp</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
+          <t>ADSL</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>EOSSTT</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>End of Study Status</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>20</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Perm</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
           <t>ADAE</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B35" t="inlineStr">
         <is>
           <t>AOCCFL</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C35" t="inlineStr">
         <is>
           <t>1st Occurrence within Subject Flag</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="E34" t="n">
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
         <v>1</v>
       </c>
-      <c r="F34" t="inlineStr">
+      <c r="F35" t="inlineStr">
         <is>
           <t>Derived</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr">
+      <c r="G35" t="inlineStr">
         <is>
           <t>Flag the first occurrence of each AEDECOD for the subject with 'Y'</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr">
+      <c r="H35" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="I34" t="inlineStr">
+      <c r="I35" t="inlineStr">
         <is>
           <t>Perm</t>
         </is>
@@ -1966,12 +2011,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2110,6 +2155,40 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>DATEFL</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Day imputed</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>DATEFL</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Month imputed</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>